<commit_message>
First iteration of buidling the full Sqlite
</commit_message>
<xml_diff>
--- a/inputs/VolumesExcel/it_IT/Paesi Bassi VOLUME 66_it_IT.xlsx
+++ b/inputs/VolumesExcel/it_IT/Paesi Bassi VOLUME 66_it_IT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/DocumentenLaptop/Programming/Github/DanielNoord/ProjectInventarisGezantschappen/inputs/VolumesExcel/it_IT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150EC954-B352-0549-9119-EFBF385D768E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B39A493E-9657-5741-A2DB-D839D9CAEC19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="28800" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2444" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2449" uniqueCount="640">
   <si>
     <t>ms341_title</t>
   </si>
@@ -2422,6 +2422,12 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>1870</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -4563,9 +4569,26 @@
       <c r="B104" t="s">
         <v>163</v>
       </c>
-      <c r="C104" s="5"/>
+      <c r="C104" s="5" t="s">
+        <v>161</v>
+      </c>
       <c r="D104">
         <v>1870</v>
+      </c>
+      <c r="E104">
+        <v>5</v>
+      </c>
+      <c r="F104">
+        <v>20</v>
+      </c>
+      <c r="G104" t="s">
+        <v>23</v>
+      </c>
+      <c r="H104" t="s">
+        <v>162</v>
+      </c>
+      <c r="I104" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="105" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>